<commit_message>
Fixes to multiple codes related to inflated uncertainties.
</commit_message>
<xml_diff>
--- a/LineClass/iter/decisions.xlsx
+++ b/LineClass/iter/decisions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\UMD\AI\as-ai\LineClass\iter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{023CAC0D-8697-4B2A-A54D-B056F76A9B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D65F4BDA-8B7B-4E8B-9460-A49358D45946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="3375" windowWidth="43920" windowHeight="17505" xr2:uid="{3B4CFF62-7D2F-4CE6-A2C0-914629AD5921}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="35520" windowHeight="17505" xr2:uid="{3B4CFF62-7D2F-4CE6-A2C0-914629AD5921}"/>
   </bookViews>
   <sheets>
     <sheet name="decisions" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">decisions!$A$1:$AE$143</definedName>
   </definedNames>
-  <calcPr calcId="0" refMode="R1C1"/>
+  <calcPr calcId="191029" refMode="R1C1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -2617,7 +2630,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>22800.4431</v>
       </c>
@@ -2697,7 +2710,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>22513.283200000002</v>
       </c>
@@ -2786,7 +2799,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>22560.4486</v>
       </c>
@@ -2961,7 +2974,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>98290.213900000002</v>
       </c>
@@ -3130,7 +3143,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>16569.385200000001</v>
       </c>
@@ -3385,7 +3398,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="11" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>97879.609700000001</v>
       </c>
@@ -3554,7 +3567,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="13" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>17331.439200000001</v>
       </c>
@@ -3637,7 +3650,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>89043.677200000006</v>
       </c>
@@ -3889,7 +3902,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>91634.468399999998</v>
       </c>
@@ -3975,7 +3988,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>97566.392699999997</v>
       </c>
@@ -4061,7 +4074,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="19" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>96377.860100000005</v>
       </c>
@@ -4313,7 +4326,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="22" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>93959.568299999999</v>
       </c>
@@ -4396,7 +4409,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>84401.620200000005</v>
       </c>
@@ -4482,7 +4495,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>102852.7668</v>
       </c>
@@ -4648,7 +4661,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="26" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>24350.653600000001</v>
       </c>
@@ -4817,7 +4830,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="28" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>56421.054499999998</v>
       </c>
@@ -5054,7 +5067,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="31" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>94935.918999999994</v>
       </c>
@@ -5137,7 +5150,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="32" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>70186.409299999999</v>
       </c>
@@ -5220,7 +5233,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>97022.822700000004</v>
       </c>
@@ -5460,7 +5473,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="36" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>27260.151600000001</v>
       </c>
@@ -5543,7 +5556,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="37" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>24593.424800000001</v>
       </c>
@@ -5620,7 +5633,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="38" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>91290.658500000005</v>
       </c>
@@ -5703,7 +5716,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="39" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>98089.89</v>
       </c>
@@ -5786,7 +5799,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="40" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>98015.090400000001</v>
       </c>
@@ -5872,7 +5885,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="41" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>95033.529699999999</v>
       </c>
@@ -6041,7 +6054,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>100444.8406</v>
       </c>
@@ -6127,7 +6140,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="44" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>94472.557100000005</v>
       </c>
@@ -6213,7 +6226,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="45" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>10255.923199999999</v>
       </c>
@@ -6370,7 +6383,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="47" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>93850.665699999998</v>
       </c>
@@ -6453,7 +6466,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="48" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>94365.236900000004</v>
       </c>
@@ -6536,7 +6549,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>89125.926600000006</v>
       </c>
@@ -6622,7 +6635,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="50" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>94081.375799999994</v>
       </c>
@@ -6791,7 +6804,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="52" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>39307.245699999999</v>
       </c>
@@ -6868,7 +6881,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="53" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>39983.802300000003</v>
       </c>
@@ -6951,7 +6964,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="54" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>38333.576200000003</v>
       </c>
@@ -7099,7 +7112,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="56" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>42117.374499999998</v>
       </c>
@@ -7185,7 +7198,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="57" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>38940.345099999999</v>
       </c>
@@ -7265,7 +7278,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="58" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>37336.752500000002</v>
       </c>
@@ -7422,7 +7435,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="60" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>42450.944600000003</v>
       </c>
@@ -7508,7 +7521,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="61" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>38333.576200000003</v>
       </c>
@@ -7668,7 +7681,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>87777.068499999994</v>
       </c>
@@ -7751,7 +7764,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="64" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>38496.7523</v>
       </c>
@@ -7840,7 +7853,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="65" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>36638.897799999999</v>
       </c>
@@ -8252,7 +8265,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="70" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>57952.534399999997</v>
       </c>
@@ -8563,7 +8576,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="74" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>56993.663200000003</v>
       </c>
@@ -8637,7 +8650,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="75" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>54261.112699999998</v>
       </c>
@@ -8723,7 +8736,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="76" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>68213.558000000005</v>
       </c>
@@ -8797,7 +8810,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="77" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>60342.597600000001</v>
       </c>
@@ -8877,7 +8890,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="78" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>55867.550300000003</v>
       </c>
@@ -8957,7 +8970,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="79" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>33491.8992</v>
       </c>
@@ -9108,7 +9121,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="81" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>54440.212899999999</v>
       </c>
@@ -9188,7 +9201,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="82" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>70254.565300000002</v>
       </c>
@@ -9271,7 +9284,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="83" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>54344.092799999999</v>
       </c>
@@ -9351,7 +9364,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="84" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>31398.824400000001</v>
       </c>
@@ -9440,7 +9453,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="85" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>67446.174199999994</v>
       </c>
@@ -9526,7 +9539,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="86" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>54703.532599999999</v>
       </c>
@@ -9692,7 +9705,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="88" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>55572.6636</v>
       </c>
@@ -9772,7 +9785,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="89" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>54607.378799999999</v>
       </c>
@@ -9852,7 +9865,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="90" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>54361.493199999997</v>
       </c>
@@ -10018,7 +10031,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="92" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>54427.654699999999</v>
       </c>
@@ -10181,7 +10194,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="94" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>38824.5412</v>
       </c>
@@ -10267,7 +10280,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="95" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>43174.807999999997</v>
       </c>
@@ -10436,7 +10449,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="97" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>54891.542500000003</v>
       </c>
@@ -10516,7 +10529,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="98" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>38282.246099999997</v>
       </c>
@@ -10596,7 +10609,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="99" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>36599.678</v>
       </c>
@@ -10753,7 +10766,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="101" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>54712.123200000002</v>
       </c>
@@ -10833,7 +10846,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="102" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>57197.535300000003</v>
       </c>
@@ -10913,7 +10926,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="103" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>55312.633600000001</v>
       </c>
@@ -10993,7 +11006,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="104" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>55387.14</v>
       </c>
@@ -11073,7 +11086,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="105" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>48601.487099999998</v>
       </c>
@@ -11159,7 +11172,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="106" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>39870.873299999999</v>
       </c>
@@ -11239,7 +11252,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="107" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>36967.159599999999</v>
       </c>
@@ -11396,7 +11409,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="109" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>26597.7664</v>
       </c>
@@ -11553,7 +11566,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="111" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>54825.9997</v>
       </c>
@@ -11633,7 +11646,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="112" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>40266.571600000003</v>
       </c>
@@ -11722,7 +11735,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="113" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>54242.751900000003</v>
       </c>
@@ -11802,7 +11815,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="114" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>23898.444599999999</v>
       </c>
@@ -11888,7 +11901,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="115" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>53932.291700000002</v>
       </c>
@@ -11977,7 +11990,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="116" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>42449.144099999998</v>
       </c>
@@ -12060,7 +12073,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="117" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>33520.092299999997</v>
       </c>
@@ -12149,7 +12162,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="118" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>32742.922900000001</v>
       </c>
@@ -12229,7 +12242,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="119" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>22524.487000000001</v>
       </c>
@@ -12392,7 +12405,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="121" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>45062.851300000002</v>
       </c>
@@ -12469,7 +12482,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="122" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>55023.862099999998</v>
       </c>
@@ -12549,7 +12562,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="123" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>23063.205099999999</v>
       </c>
@@ -12638,7 +12651,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="124" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>44931.700900000003</v>
       </c>
@@ -12727,7 +12740,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="125" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>54202.265700000004</v>
       </c>
@@ -12807,7 +12820,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="126" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>45062.851300000002</v>
       </c>
@@ -12884,7 +12897,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="127" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>40169.222600000001</v>
       </c>
@@ -12973,7 +12986,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="128" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>33207.6636</v>
       </c>
@@ -13062,7 +13075,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="129" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>32105.398000000001</v>
       </c>
@@ -13225,7 +13238,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="131" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>39447.448700000001</v>
       </c>
@@ -13314,7 +13327,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="132" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>39307.245699999999</v>
       </c>
@@ -13391,7 +13404,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="133" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>22665.3832</v>
       </c>
@@ -13850,7 +13863,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="139" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>38726.351699999999</v>
       </c>
@@ -14013,7 +14026,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="141" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>26157.9568</v>
       </c>
@@ -14093,7 +14106,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="142" spans="1:31" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>18768.147199999999</v>
       </c>
@@ -14252,11 +14265,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AE143" xr:uid="{273CACE9-914D-4F0F-BB6B-3C5D2CC52055}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="900"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="29">
       <filters>
         <filter val="review"/>

</xml_diff>